<commit_message>
cambio de menbrete 2026
</commit_message>
<xml_diff>
--- a/assets/plantilla_camion.xlsx
+++ b/assets/plantilla_camion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://intigobar-my.sharepoint.com/personal/psiklosi_inti_gob_ar/Documents/extract_camiones/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="310" documentId="11_A652BFD88C009AA27A2DEFB33DEEFBFD99302097" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3B3917E-09D4-4B3E-BDB9-ADE8070295BA}"/>
+  <xr:revisionPtr revIDLastSave="332" documentId="11_A652BFD88C009AA27A2DEFB33DEEFBFD99302097" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7198CD60-8617-4DAC-AFF9-52BC662B30DA}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="718" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="718" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="datos vpe" sheetId="13" r:id="rId1"/>
@@ -341,7 +341,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="747">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="744">
   <si>
     <t>Mendoza</t>
   </si>
@@ -2411,24 +2411,9 @@
     <t xml:space="preserve">Jefe de mantenimiento </t>
   </si>
   <si>
-    <t>(a) N03474</t>
-  </si>
-  <si>
-    <t>(a) N03475</t>
-  </si>
-  <si>
-    <t>(a) B79341, B79342 (05/11/25)</t>
-  </si>
-  <si>
-    <t>(a) B739443, B79344 (05/11/25)</t>
-  </si>
-  <si>
     <t>Verificado</t>
   </si>
   <si>
-    <t>(a) 1104924 (05/11/25)</t>
-  </si>
-  <si>
     <t>Campo</t>
   </si>
   <si>
@@ -2616,6 +2601,12 @@
   </si>
   <si>
     <t>30-71679479-9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(a) </t>
+  </si>
+  <si>
+    <t>(a)</t>
   </si>
 </sst>
 </file>
@@ -8063,20 +8054,20 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>804012</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>95371</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6624" name="Imagen 1">
+        <xdr:cNvPr id="2" name="Imagen 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-0000E0190000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{03A28D59-2CDB-6740-7380-D1C939B767F3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -8086,24 +8077,62 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
+      <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="6738087" cy="1085850"/>
+          <a:off x="0" y="1"/>
+          <a:ext cx="6781800" cy="1238370"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>790575</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>39142</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6EE509D4-637C-48AE-F5D0-50306030EA65}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="28575" y="10296525"/>
+          <a:ext cx="6696075" cy="1029742"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -8113,56 +8142,6 @@
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>614813</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="7646" name="Imagen 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-0000DE1D0000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="6910838" cy="1333500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -8213,6 +8192,94 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>619125</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>119721</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BDB206BF-0B72-B990-CE2D-44040B3B19DC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="1"/>
+          <a:ext cx="6915150" cy="1262720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>609600</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>109467</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{06AC937D-A6A7-13C4-AD1D-3BF66ADF4BC0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="10001250"/>
+          <a:ext cx="6905625" cy="1061967"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -8226,17 +8293,17 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>249247</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>476250</xdr:rowOff>
+      <xdr:rowOff>466725</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
+        <xdr:cNvPr id="3" name="Imagen 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C4544F10-F816-44B2-82F1-85A6F063B953}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9B84A09-4D2B-4F6B-8706-417B77DC8242}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -8246,22 +8313,19 @@
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
+      <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="5726122" cy="1104900"/>
+          <a:ext cx="5981700" cy="1095375"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
         <a:ln>
-          <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </xdr:spPr>
@@ -8793,39 +8857,39 @@
   <sheetData>
     <row r="1" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="754" t="s">
-        <v>684</v>
+        <v>679</v>
       </c>
       <c r="B1" s="754" t="s">
-        <v>685</v>
+        <v>680</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="756" t="s">
-        <v>741</v>
+        <v>736</v>
       </c>
       <c r="B2" s="759">
-        <v>45658</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="756" t="s">
-        <v>686</v>
+        <v>681</v>
       </c>
       <c r="B3" s="758" t="s">
-        <v>735</v>
+        <v>730</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="756" t="s">
-        <v>687</v>
+        <v>682</v>
       </c>
       <c r="B4" s="757" t="s">
-        <v>736</v>
+        <v>731</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="756" t="s">
-        <v>688</v>
+        <v>683</v>
       </c>
       <c r="B5" s="757" t="s">
         <v>30</v>
@@ -8833,23 +8897,23 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="756" t="s">
-        <v>689</v>
+        <v>684</v>
       </c>
       <c r="B6" s="757" t="s">
-        <v>690</v>
+        <v>685</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="756" t="s">
-        <v>691</v>
+        <v>686</v>
       </c>
       <c r="B7" s="757" t="s">
-        <v>692</v>
+        <v>687</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="756" t="s">
-        <v>693</v>
+        <v>688</v>
       </c>
       <c r="B8" s="757" t="s">
         <v>30</v>
@@ -8857,7 +8921,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="756" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="B9" s="757" t="s">
         <v>30</v>
@@ -8865,23 +8929,23 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="756" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="B10" s="757" t="s">
-        <v>696</v>
+        <v>691</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="756" t="s">
-        <v>697</v>
+        <v>692</v>
       </c>
       <c r="B11" s="757" t="s">
-        <v>698</v>
+        <v>693</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="756" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="B12" s="757" t="s">
         <v>0</v>
@@ -8889,7 +8953,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="756" t="s">
-        <v>700</v>
+        <v>695</v>
       </c>
       <c r="B13" s="757" t="s">
         <v>1</v>
@@ -8897,42 +8961,42 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="756" t="s">
-        <v>701</v>
+        <v>696</v>
       </c>
       <c r="B14" s="757" t="s">
-        <v>702</v>
+        <v>697</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="756" t="s">
-        <v>703</v>
+        <v>698</v>
       </c>
       <c r="B15" s="757" t="s">
-        <v>704</v>
+        <v>699</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="756" t="s">
-        <v>705</v>
+        <v>700</v>
       </c>
       <c r="B16" s="757" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="756" t="s">
-        <v>707</v>
+        <v>702</v>
       </c>
       <c r="B17" s="757" t="s">
-        <v>737</v>
+        <v>732</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="756" t="s">
-        <v>708</v>
+        <v>703</v>
       </c>
       <c r="B18" s="757" t="s">
-        <v>709</v>
+        <v>704</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -8945,39 +9009,39 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="756" t="s">
-        <v>710</v>
+        <v>705</v>
       </c>
       <c r="B20" s="757" t="s">
-        <v>711</v>
+        <v>706</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="756" t="s">
-        <v>712</v>
+        <v>707</v>
       </c>
       <c r="B21" s="757" t="s">
-        <v>713</v>
+        <v>708</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="756" t="s">
-        <v>714</v>
+        <v>709</v>
       </c>
       <c r="B22" s="757" t="s">
-        <v>715</v>
+        <v>710</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="756" t="s">
-        <v>716</v>
+        <v>711</v>
       </c>
       <c r="B23" s="757" t="s">
-        <v>711</v>
+        <v>706</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="756" t="s">
-        <v>717</v>
+        <v>712</v>
       </c>
       <c r="B24" s="757" t="s">
         <v>3</v>
@@ -8985,23 +9049,23 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="756" t="s">
-        <v>718</v>
+        <v>713</v>
       </c>
       <c r="B25" s="757" t="s">
-        <v>719</v>
+        <v>714</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="756" t="s">
-        <v>720</v>
+        <v>715</v>
       </c>
       <c r="B26" s="757" t="s">
-        <v>721</v>
+        <v>716</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="756" t="s">
-        <v>722</v>
+        <v>717</v>
       </c>
       <c r="B27" s="757" t="s">
         <v>4</v>
@@ -9009,47 +9073,47 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="756" t="s">
-        <v>723</v>
+        <v>718</v>
       </c>
       <c r="B28" s="757" t="s">
-        <v>702</v>
+        <v>697</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="756" t="s">
-        <v>724</v>
+        <v>719</v>
       </c>
       <c r="B29" s="757" t="s">
-        <v>704</v>
+        <v>699</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="756" t="s">
-        <v>725</v>
+        <v>720</v>
       </c>
       <c r="B30" s="757" t="s">
-        <v>726</v>
+        <v>721</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="756" t="s">
-        <v>727</v>
+        <v>722</v>
       </c>
       <c r="B31" s="757" t="s">
-        <v>738</v>
+        <v>733</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="756" t="s">
-        <v>728</v>
+        <v>723</v>
       </c>
       <c r="B32" s="757" t="s">
-        <v>729</v>
+        <v>724</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="756" t="s">
-        <v>730</v>
+        <v>725</v>
       </c>
       <c r="B33" s="757" t="s">
         <v>673</v>
@@ -9057,18 +9121,18 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="756" t="s">
-        <v>731</v>
+        <v>726</v>
       </c>
       <c r="B34" s="757" t="s">
-        <v>732</v>
+        <v>727</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="756" t="s">
-        <v>733</v>
+        <v>728</v>
       </c>
       <c r="B35" s="757" t="s">
-        <v>734</v>
+        <v>729</v>
       </c>
     </row>
   </sheetData>
@@ -9390,7 +9454,7 @@
     <row r="15" spans="1:44" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1046" t="str">
         <f>Informe!A15</f>
-        <v>Precintos Nº: Placa identificatoria del receptor (a) N03475, Placa identificatoria del indicador (a) N03474, Indicador (a) B79341, B79342 (05/11/25), Caja de ecualización (a) B739443, B79344 (05/11/25) y Verificado (a) 1104924 (05/11/25).</v>
+        <v>Precintos Nº: Placa identificatoria del receptor (a) , Placa identificatoria del indicador (a) , Indicador (a), Caja de ecualización (a) y Verificado (a).</v>
       </c>
       <c r="B15" s="1009"/>
       <c r="C15" s="1009"/>
@@ -9573,7 +9637,7 @@
       <c r="C24" s="1045"/>
       <c r="D24" s="1044" t="str">
         <f>Informe!D28</f>
-        <v>1 de enero de 2025</v>
+        <v>1 de marzo de 2026</v>
       </c>
       <c r="E24" s="1045"/>
       <c r="F24" s="1045"/>
@@ -9629,7 +9693,7 @@
       <c r="C25" s="1045"/>
       <c r="D25" s="1044">
         <f ca="1">TODAY()</f>
-        <v>46009</v>
+        <v>46084</v>
       </c>
       <c r="E25" s="1045"/>
       <c r="F25" s="1045"/>
@@ -12032,7 +12096,7 @@
       <c r="D4" s="1093"/>
       <c r="E4" s="1092" t="str">
         <f>CONCATENATE("Fecha: ", IF(COUNTA('Identificación del Instrumento'!J2)=0,"",'Identificación del Instrumento'!J2))</f>
-        <v>Fecha: 1 de enero de 2025</v>
+        <v>Fecha: 1 de marzo de 2026</v>
       </c>
       <c r="F4" s="1093"/>
       <c r="G4" s="1093"/>
@@ -16054,7 +16118,7 @@
       </c>
       <c r="J2" s="815" t="str">
         <f>CONCATENATE(D3, " de ",E3, " de ",F3)</f>
-        <v>1 de enero de 2025</v>
+        <v>1 de marzo de 2026</v>
       </c>
       <c r="K2" s="765"/>
       <c r="L2" s="678"/>
@@ -16072,11 +16136,11 @@
       </c>
       <c r="E3" s="677" t="str">
         <f>IFERROR(TEXT(_xlfn.XLOOKUP("Fecha estimada de verificación",'datos vpe'!A:A,'datos vpe'!B:B,""),"mmmm"),"")</f>
-        <v>enero</v>
+        <v>marzo</v>
       </c>
       <c r="F3" s="676">
         <f>IFERROR(YEAR(_xlfn.XLOOKUP("Fecha estimada de verificación",'datos vpe'!A:A,'datos vpe'!B:B,"")),"")</f>
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="H3" s="675"/>
       <c r="I3" s="679" t="s">
@@ -16084,7 +16148,7 @@
       </c>
       <c r="J3" s="815" t="str">
         <f>CONCATENATE(D3, " de ",E3, " de ",F3+2)</f>
-        <v>1 de enero de 2027</v>
+        <v>1 de marzo de 2028</v>
       </c>
       <c r="K3" s="765"/>
       <c r="L3" s="675"/>
@@ -16834,7 +16898,7 @@
         <v>84</v>
       </c>
       <c r="J35" s="743" t="s">
-        <v>746</v>
+        <v>741</v>
       </c>
       <c r="N35" s="25">
         <v>2</v>
@@ -16881,10 +16945,10 @@
       </c>
       <c r="G37" s="800"/>
       <c r="I37" s="743" t="s">
-        <v>739</v>
+        <v>734</v>
       </c>
       <c r="J37" s="743" t="s">
-        <v>740</v>
+        <v>735</v>
       </c>
       <c r="P37" s="212" t="s">
         <v>90</v>
@@ -17796,7 +17860,7 @@
       <c r="J6" s="783"/>
       <c r="K6" s="912" t="str">
         <f>'Identificación del Instrumento'!J2</f>
-        <v>1 de enero de 2025</v>
+        <v>1 de marzo de 2026</v>
       </c>
       <c r="L6" s="858"/>
       <c r="M6" s="105"/>
@@ -18514,17 +18578,17 @@
       <c r="R22" s="116"/>
       <c r="S22" s="116"/>
       <c r="AC22" s="243" t="s">
-        <v>742</v>
+        <v>737</v>
       </c>
       <c r="AD22" s="241" t="s">
-        <v>743</v>
+        <v>738</v>
       </c>
       <c r="AE22" s="242" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="AF22" s="242"/>
       <c r="AG22" s="761" t="s">
-        <v>745</v>
+        <v>740</v>
       </c>
       <c r="AH22" s="109"/>
       <c r="AI22" s="110"/>
@@ -33255,7 +33319,7 @@
       <c r="H1" s="942"/>
       <c r="J1" s="336" t="str">
         <f>CONCATENATE("En la localidad de ",'Identificación del Instrumento'!$D$4,", provincia de ",'Identificación del Instrumento'!$D$5,", siendo las ",$J$18," horas del día ",'Identificación del Instrumento'!J2,", en virtud de la solicitud presentada por la firma ",'Identificación del Instrumento'!$C$14,", conforme a lo establecido en la Resolución Nº 611/2019 de la SECRETARÍA DE COMERCIO INTERIOR y sus modificatorias, el ",$T$18,", ",$T$19,", habilitado por el INSTITUTO NACIONAL DE TECNOLOGÍA INDUSTRIAL (I.N.T.I.), con credencial acreditante N° ",$T$20,", que en este acto se exhibe")</f>
-        <v>En la localidad de COSTA DE ARAUJO, provincia de Mendoza, siendo las 15:30 horas del día 1 de enero de 2025, en virtud de la solicitud presentada por la firma Marolio S.A., conforme a lo establecido en la Resolución Nº 611/2019 de la SECRETARÍA DE COMERCIO INTERIOR y sus modificatorias, el Tco. Pablo Javier Siklosi A., D.N.I. N° 24.705.518, habilitado por el INSTITUTO NACIONAL DE TECNOLOGÍA INDUSTRIAL (I.N.T.I.), con credencial acreditante N° 96, que en este acto se exhibe</v>
+        <v>En la localidad de COSTA DE ARAUJO, provincia de Mendoza, siendo las 15:30 horas del día 1 de marzo de 2026, en virtud de la solicitud presentada por la firma Marolio S.A., conforme a lo establecido en la Resolución Nº 611/2019 de la SECRETARÍA DE COMERCIO INTERIOR y sus modificatorias, el Tco. Pablo Javier Siklosi A., D.N.I. N° 24.705.518, habilitado por el INSTITUTO NACIONAL DE TECNOLOGÍA INDUSTRIAL (I.N.T.I.), con credencial acreditante N° 96, que en este acto se exhibe</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -33461,7 +33525,7 @@
     <row r="18" spans="1:22" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="960" t="str">
         <f>IF($J$29=6,CONCATENATE($J$1,$J$2),"¡Completar datos del acta!")</f>
-        <v>En la localidad de COSTA DE ARAUJO, provincia de Mendoza, siendo las 15:30 horas del día 1 de enero de 2025, en virtud de la solicitud presentada por la firma Marolio S.A., conforme a lo establecido en la Resolución Nº 611/2019 de la SECRETARÍA DE COMERCIO INTERIOR y sus modificatorias, el Tco. Pablo Javier Siklosi A., D.N.I. N° 24.705.518, habilitado por el INSTITUTO NACIONAL DE TECNOLOGÍA INDUSTRIAL (I.N.T.I.), con credencial acreditante N° 96, que en este acto se exhibe, en ejecución y en ejercicio de las facultades conferidas por la ley Nº 19.511, el Decreto Reglamentario N° 960/2017, la Resolución Nº 611/2019 y sus modifiatorias, procede a hacerse presente en Zona de pesaje de la firma citada, ubicada en RUTA PROVINCIAL Nº 20 S/N, siendo recibido por quien acredita ser Sr. Nievas Aldo Dario; D.N.I. Nº 21.038.713, quien se desempeña en la firma como Jefe de mantenimiento  y suscribe este instrumento en prueba de conformidad.</v>
+        <v>En la localidad de COSTA DE ARAUJO, provincia de Mendoza, siendo las 15:30 horas del día 1 de marzo de 2026, en virtud de la solicitud presentada por la firma Marolio S.A., conforme a lo establecido en la Resolución Nº 611/2019 de la SECRETARÍA DE COMERCIO INTERIOR y sus modificatorias, el Tco. Pablo Javier Siklosi A., D.N.I. N° 24.705.518, habilitado por el INSTITUTO NACIONAL DE TECNOLOGÍA INDUSTRIAL (I.N.T.I.), con credencial acreditante N° 96, que en este acto se exhibe, en ejecución y en ejercicio de las facultades conferidas por la ley Nº 19.511, el Decreto Reglamentario N° 960/2017, la Resolución Nº 611/2019 y sus modifiatorias, procede a hacerse presente en Zona de pesaje de la firma citada, ubicada en RUTA PROVINCIAL Nº 20 S/N, siendo recibido por quien acredita ser Sr. Nievas Aldo Dario; D.N.I. Nº 21.038.713, quien se desempeña en la firma como Jefe de mantenimiento  y suscribe este instrumento en prueba de conformidad.</v>
       </c>
       <c r="B18" s="786"/>
       <c r="C18" s="786"/>
@@ -34066,7 +34130,7 @@
       <c r="O47" s="455"/>
       <c r="P47" s="455"/>
     </row>
-    <row r="48" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:16" ht="4.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="786"/>
       <c r="B48" s="786"/>
       <c r="C48" s="786"/>
@@ -34092,7 +34156,7 @@
       <c r="O49" s="455"/>
       <c r="P49" s="455"/>
     </row>
-    <row r="50" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="786"/>
       <c r="B50" s="786"/>
       <c r="C50" s="786"/>
@@ -34115,7 +34179,7 @@
       <c r="G51" s="786"/>
       <c r="H51" s="786"/>
     </row>
-    <row r="52" spans="1:16" s="395" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:16" s="395" customFormat="1" ht="3" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="576"/>
       <c r="B52" s="576"/>
       <c r="C52" s="576"/>
@@ -34223,7 +34287,7 @@
       <c r="G60" s="576"/>
       <c r="H60" s="576"/>
     </row>
-    <row r="61" spans="1:16" s="505" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:16" s="505" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="576"/>
       <c r="B61" s="576"/>
       <c r="C61" s="576"/>
@@ -34588,7 +34652,7 @@
       </c>
       <c r="B13" s="981" t="str">
         <f>IF(ISBLANK('Identificación del Instrumento'!J2),"",'Identificación del Instrumento'!J2)</f>
-        <v>1 de enero de 2025</v>
+        <v>1 de marzo de 2026</v>
       </c>
       <c r="C13" s="841"/>
       <c r="D13" s="841"/>
@@ -34845,7 +34909,7 @@
       </c>
       <c r="D24" s="966"/>
       <c r="E24" s="988" t="s">
-        <v>679</v>
+        <v>742</v>
       </c>
       <c r="F24" s="880"/>
       <c r="G24" s="880"/>
@@ -34864,7 +34928,7 @@
       </c>
       <c r="S24" s="229" t="str">
         <f>IF(ISBLANK(E24),"",IF(ISBLANK(E25),CONCATENATE("",B24," ",C24, " ",E24),CONCATENATE("",B24," ",C24," ",E24)))</f>
-        <v>Placa identificatoria del receptor (a) N03475</v>
+        <v xml:space="preserve">Placa identificatoria del receptor (a) </v>
       </c>
     </row>
     <row r="25" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
@@ -34875,7 +34939,7 @@
       </c>
       <c r="D25" s="966"/>
       <c r="E25" s="968" t="s">
-        <v>678</v>
+        <v>742</v>
       </c>
       <c r="F25" s="769"/>
       <c r="G25" s="769"/>
@@ -34890,7 +34954,7 @@
       <c r="O25" s="228"/>
       <c r="S25" s="230" t="str">
         <f>IF(ISBLANK(E25),"",IF(ISBLANK(E26),CONCATENATE(" y ",B24," ",C25," ",E25),CONCATENATE(", ",B24," ",C25," ",E25)))</f>
-        <v>, Placa identificatoria del indicador (a) N03474</v>
+        <v xml:space="preserve">, Placa identificatoria del indicador (a) </v>
       </c>
     </row>
     <row r="26" spans="1:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -34901,7 +34965,7 @@
       <c r="C26" s="769"/>
       <c r="D26" s="800"/>
       <c r="E26" s="968" t="s">
-        <v>680</v>
+        <v>743</v>
       </c>
       <c r="F26" s="769"/>
       <c r="G26" s="769"/>
@@ -34916,7 +34980,7 @@
       <c r="O26" s="228"/>
       <c r="S26" s="230" t="str">
         <f>IF(ISBLANK(E26),"",IF(ISBLANK(E27),CONCATENATE(", ",B26, " ",E26),CONCATENATE(", ",B26," ",E26)))</f>
-        <v>, Indicador (a) B79341, B79342 (05/11/25)</v>
+        <v>, Indicador (a)</v>
       </c>
     </row>
     <row r="27" spans="1:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -34927,7 +34991,7 @@
       <c r="C27" s="769"/>
       <c r="D27" s="800"/>
       <c r="E27" s="968" t="s">
-        <v>681</v>
+        <v>743</v>
       </c>
       <c r="F27" s="769"/>
       <c r="G27" s="769"/>
@@ -34942,18 +35006,18 @@
       <c r="O27" s="228"/>
       <c r="S27" s="230" t="str">
         <f>IF(ISBLANK(E27),"",IF(ISBLANK(E28),CONCATENATE(", ",B27, " ",E27),CONCATENATE(", ",B27," ",E27)))</f>
-        <v>, Caja de ecualización (a) B739443, B79344 (05/11/25)</v>
+        <v>, Caja de ecualización (a)</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="380"/>
       <c r="B28" s="967" t="s">
-        <v>682</v>
+        <v>678</v>
       </c>
       <c r="C28" s="769"/>
       <c r="D28" s="800"/>
       <c r="E28" s="971" t="s">
-        <v>683</v>
+        <v>743</v>
       </c>
       <c r="F28" s="769"/>
       <c r="G28" s="800"/>
@@ -34968,7 +35032,7 @@
       <c r="O28" s="228"/>
       <c r="S28" s="230" t="str">
         <f t="shared" ref="S28:S46" si="0">IF(ISBLANK(E28),"",IF(ISBLANK(E29),CONCATENATE(" y ",B28, " ",E28),CONCATENATE(", ",B28," ",E28)))</f>
-        <v xml:space="preserve"> y Verificado (a) 1104924 (05/11/25)</v>
+        <v xml:space="preserve"> y Verificado (a)</v>
       </c>
     </row>
     <row r="29" spans="1:19" ht="33" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -35327,7 +35391,7 @@
       <c r="O49" s="408"/>
       <c r="S49" s="231" t="str">
         <f>CONCATENATE(S24,S25,S26,S27,S28,S29,S30,S31,S32,S33,S34,S35,S36,S37,S38,S39,S40,S41,S42,S43,S44,S45,S46,S47)</f>
-        <v>Placa identificatoria del receptor (a) N03475, Placa identificatoria del indicador (a) N03474, Indicador (a) B79341, B79342 (05/11/25), Caja de ecualización (a) B739443, B79344 (05/11/25) y Verificado (a) 1104924 (05/11/25)</v>
+        <v>Placa identificatoria del receptor (a) , Placa identificatoria del indicador (a) , Indicador (a), Caja de ecualización (a) y Verificado (a)</v>
       </c>
     </row>
     <row r="50" spans="1:19" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -36090,7 +36154,7 @@
     <row r="15" spans="1:44" ht="53.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="824" t="str">
         <f>CONCATENATE("Precintos Nº: ",'Acta Precintos'!S49,".")</f>
-        <v>Precintos Nº: Placa identificatoria del receptor (a) N03475, Placa identificatoria del indicador (a) N03474, Indicador (a) B79341, B79342 (05/11/25), Caja de ecualización (a) B739443, B79344 (05/11/25) y Verificado (a) 1104924 (05/11/25).</v>
+        <v>Precintos Nº: Placa identificatoria del receptor (a) , Placa identificatoria del indicador (a) , Indicador (a), Caja de ecualización (a) y Verificado (a).</v>
       </c>
       <c r="B15" s="995"/>
       <c r="C15" s="995"/>
@@ -36477,7 +36541,7 @@
       <c r="C28" s="995"/>
       <c r="D28" s="1006" t="str">
         <f>'Identificación del Instrumento'!J2</f>
-        <v>1 de enero de 2025</v>
+        <v>1 de marzo de 2026</v>
       </c>
       <c r="E28" s="997"/>
       <c r="F28" s="995"/>
@@ -36494,7 +36558,7 @@
       <c r="C29" s="995"/>
       <c r="D29" s="1006">
         <f ca="1">TODAY()</f>
-        <v>46009</v>
+        <v>46084</v>
       </c>
       <c r="E29" s="997"/>
       <c r="F29" s="995"/>
@@ -36511,7 +36575,7 @@
       <c r="C30" s="995"/>
       <c r="D30" s="1006" t="str">
         <f>'Identificación del Instrumento'!J3</f>
-        <v>1 de enero de 2027</v>
+        <v>1 de marzo de 2028</v>
       </c>
       <c r="E30" s="997"/>
       <c r="F30" s="995"/>
@@ -37562,7 +37626,7 @@
       <c r="G1" s="841"/>
       <c r="H1" s="1025">
         <f ca="1">TODAY()</f>
-        <v>46009</v>
+        <v>46084</v>
       </c>
       <c r="I1" s="841"/>
     </row>
@@ -37573,7 +37637,7 @@
       <c r="G2" s="841"/>
       <c r="H2" s="1024" t="str">
         <f>+Informe!D30</f>
-        <v>1 de enero de 2027</v>
+        <v>1 de marzo de 2028</v>
       </c>
       <c r="I2" s="841"/>
     </row>
@@ -37740,7 +37804,7 @@
       </c>
       <c r="B29" t="str">
         <f>Informe!D28</f>
-        <v>1 de enero de 2025</v>
+        <v>1 de marzo de 2026</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -37792,7 +37856,7 @@
       </c>
       <c r="B36" s="1026" t="str">
         <f>+Informe!A15</f>
-        <v>Precintos Nº: Placa identificatoria del receptor (a) N03475, Placa identificatoria del indicador (a) N03474, Indicador (a) B79341, B79342 (05/11/25), Caja de ecualización (a) B739443, B79344 (05/11/25) y Verificado (a) 1104924 (05/11/25).</v>
+        <v>Precintos Nº: Placa identificatoria del receptor (a) , Placa identificatoria del indicador (a) , Indicador (a), Caja de ecualización (a) y Verificado (a).</v>
       </c>
       <c r="C36" s="841"/>
       <c r="D36" s="841"/>
@@ -37911,7 +37975,7 @@
       <c r="H3" s="573"/>
       <c r="N3" t="str">
         <f>CONCATENATE("En la localidad de ",'Identificación del Instrumento'!$D$4,", provincia de ",'Identificación del Instrumento'!$D$5,", siendo las ",$J$18," horas del día ",TEXT('Identificación del Instrumento'!J2,"d/mm/yyyy"),", en virtud de la solicitud y declaración jurada presentada por la firma ",'Identificación del Instrumento'!$C$14,", conforme el punto ",$J$27,"  de la Resolución Nº 611/2019 de la SECRETARÍA DE COMERCIO INTERIOR, el ",$T$18,", ",$T$19,", habilitado por el INSTITUTO NACIONAL DE TECNOLOGÍA INDUSTRIAL (I.N.T.I.), con credencial acreditante N° ",$T$20,", que en este acto se exhibe")</f>
-        <v>En la localidad de COSTA DE ARAUJO, provincia de Mendoza, siendo las 15:00 horas del día 1 de enero de 2025, en virtud de la solicitud y declaración jurada presentada por la firma Marolio S.A., conforme el punto 1 del Cap. III del Anexo I  de la Resolución Nº 611/2019 de la SECRETARÍA DE COMERCIO INTERIOR, el Tco. Pablo Javier Siklosi A., D.N.I. N° 24.705.518, habilitado por el INSTITUTO NACIONAL DE TECNOLOGÍA INDUSTRIAL (I.N.T.I.), con credencial acreditante N° 96, que en este acto se exhibe</v>
+        <v>En la localidad de COSTA DE ARAUJO, provincia de Mendoza, siendo las 15:00 horas del día 1 de marzo de 2026, en virtud de la solicitud y declaración jurada presentada por la firma Marolio S.A., conforme el punto 1 del Cap. III del Anexo I  de la Resolución Nº 611/2019 de la SECRETARÍA DE COMERCIO INTERIOR, el Tco. Pablo Javier Siklosi A., D.N.I. N° 24.705.518, habilitado por el INSTITUTO NACIONAL DE TECNOLOGÍA INDUSTRIAL (I.N.T.I.), con credencial acreditante N° 96, que en este acto se exhibe</v>
       </c>
     </row>
     <row r="4" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -38178,7 +38242,7 @@
     <row r="18" spans="1:31" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="960" t="str">
         <f>IF($J$28=6,CONCATENATE($N$3,$N$4),"¡Completar datos del acta!")</f>
-        <v>En la localidad de COSTA DE ARAUJO, provincia de Mendoza, siendo las 15:00 horas del día 1 de enero de 2025, en virtud de la solicitud y declaración jurada presentada por la firma Marolio S.A., conforme el punto 1 del Cap. III del Anexo I  de la Resolución Nº 611/2019 de la SECRETARÍA DE COMERCIO INTERIOR, el Tco. Pablo Javier Siklosi A., D.N.I. N° 24.705.518, habilitado por el INSTITUTO NACIONAL DE TECNOLOGÍA INDUSTRIAL (I.N.T.I.), con credencial acreditante N° 96, que en este acto se exhibe, en ejecución y en ejercicio de las facultades conferidas por la ley Nº 19.511,  el inciso l) del Artículo 2 del Decreto Reglamentario N° 960/2017, el inciso a) del Artículo 1 de la Resolución E 8/2018 del 10 de enero del 2018 de la Secretaría de Comercio y los puntos 1 del Cap. I y 1 del Cap. III  ambos del Anexo I la citada Resolución Nº 611/2019, procede a hacerse presente en Zona de pesaje de la firma citada, ubicada en RUTA PROVINCIAL Nº 20 S/N, de la localidad de COSTA DE ARAUJO, provincia de Mendoza, siendo recibido por quien acredita ser Sr. Nievas Aldo Dario, D.N.I. Nº 21.038.713, quien se desempeña en la firma como Jefe de mantenimiento  y suscribe este instrumento en prueba de conformidad.</v>
+        <v>En la localidad de COSTA DE ARAUJO, provincia de Mendoza, siendo las 15:00 horas del día 1 de marzo de 2026, en virtud de la solicitud y declaración jurada presentada por la firma Marolio S.A., conforme el punto 1 del Cap. III del Anexo I  de la Resolución Nº 611/2019 de la SECRETARÍA DE COMERCIO INTERIOR, el Tco. Pablo Javier Siklosi A., D.N.I. N° 24.705.518, habilitado por el INSTITUTO NACIONAL DE TECNOLOGÍA INDUSTRIAL (I.N.T.I.), con credencial acreditante N° 96, que en este acto se exhibe, en ejecución y en ejercicio de las facultades conferidas por la ley Nº 19.511,  el inciso l) del Artículo 2 del Decreto Reglamentario N° 960/2017, el inciso a) del Artículo 1 de la Resolución E 8/2018 del 10 de enero del 2018 de la Secretaría de Comercio y los puntos 1 del Cap. I y 1 del Cap. III  ambos del Anexo I la citada Resolución Nº 611/2019, procede a hacerse presente en Zona de pesaje de la firma citada, ubicada en RUTA PROVINCIAL Nº 20 S/N, de la localidad de COSTA DE ARAUJO, provincia de Mendoza, siendo recibido por quien acredita ser Sr. Nievas Aldo Dario, D.N.I. Nº 21.038.713, quien se desempeña en la firma como Jefe de mantenimiento  y suscribe este instrumento en prueba de conformidad.</v>
       </c>
       <c r="B18" s="786"/>
       <c r="C18" s="786"/>

</xml_diff>